<commit_message>
v0.00.001 feat(SHBS-17): USB-C-Buchse auf 12401598E4#2A umgestellt, Ersatz fuer PS1 vorgeschlagen
J1 und J_PWR1: Die abgekuendigte Amphenol 12401548E4#2A ist durch den
Nachfolger 12401598E4#2A ersetzt. Die neue Buchse ist nicht pad-kompatibel:
die B-Reihe ist SMD statt THT. Padbild aus dem Amphenol-STEP-Modell
ermittelt, es deckt sich mit dem KiCad-Footprint der Schwester
12401610E4-2A; uebernommen als shbs_power:USB_C_Receptacle_Amphenol_
12401598E4-2A. Schaltplan, Symbol-Cache und power.kicad_sym umgestellt,
ERC 0 Fehler.

PS1: Diodes AP3211KTR-G1 als pinkompatibler Ersatz fuer den MP2359
(NRND, ohne Lager) in der Stueckliste vorgeschlagen, Schaltplan noch
unveraendert. Alle 46 Positionen lieferbar, 47,78 EUR pro Baugruppe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
+++ b/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
@@ -546,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Quelle: PCB/BasisStation/*.kicad_sch · Stand 2026-09-23 · 46 Positionen · 78 Bauteile</t>
+          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-23 · 46 Positionen · 78 Bauteile</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>12401548E4-2A</t>
+          <t>12401598E4-2A</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>shbs_power:USB_C_Receptacle_Amphenol_12401548E4-2A</t>
+          <t>shbs_power:USB_C_Receptacle_Amphenol_12401598E4-2A</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -3099,16 +3099,12 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="V29" s="10" t="inlineStr">
-        <is>
-          <t>Vorschlag</t>
-        </is>
-      </c>
-      <c r="W29" s="5" t="inlineStr">
-        <is>
-          <t>Ersatz für 12401548E4#2A (abgekündigt). Nachfolger laut Mouser für die abgekündigte 12401548E4#2A; laut DigiKey gleiche Bauart (24-polig, Hybrid SMD/THT, rechtwinklig), zusätzlich Führungsstifte. Vor Übernahme Zeichnung gegen Footprint prüfen. Nach Freigabe als Feld in den Schaltplan übernehmen.</t>
-        </is>
-      </c>
+      <c r="V29" s="4" t="inlineStr">
+        <is>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -3345,44 +3341,44 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Monolithic Power Systems</t>
+          <t>Diodes Incorporated</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>MP2359DJ-LF-Z</t>
+          <t>AP3211KTR-G1</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>946-MP2359DJLFZ</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="K32" s="11" t="n">
-        <v>0</v>
+          <t>621-AP3211KTR-G1</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>18260</v>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>1589-1889-1-ND</t>
+          <t>AP3211KTR-G1DICT-ND</t>
         </is>
       </c>
       <c r="M32" s="6" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="N32" s="11" t="n">
-        <v>0</v>
+        <v>0.47</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>32678</v>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>Not Recommended for New Designs</t>
-        </is>
-      </c>
-      <c r="P32" s="11" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
+          <t>Aktiv</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q32" s="8">
@@ -3408,14 +3404,14 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="V32" s="11" t="inlineStr">
-        <is>
-          <t>Ersatz nötig</t>
+      <c r="V32" s="10" t="inlineStr">
+        <is>
+          <t>Vorschlag</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
         <is>
-          <t>Abgekündigt (Mouser: Not Recommended for New Designs; DigiKey: Nicht für Neukonstruktionen) — Ersatztyp wählen. Bei keinem Distributor ab Lager lieferbar (Lager DigiKey: 0) — Lieferzeit anfragen oder Ersatz wählen.</t>
+          <t>Ersatz für MP2359DJ-LF-Z (abgekündigt). Pinkompatibel (1 BS, 2 GND, 3 FB, 4 EN, 5 IN, 6 SW), SOT-23-6 passt auf den Footprint MP2359DJ, VFB 0,81 V (R17/R18 bleiben), 1,4 MHz, asynchron mit D11, 1,5 A. Prüfen: Strombegrenzung 1,8–2,4 A gegen den Sättigungsstrom von L1. Nach Freigabe als Feld in den Schaltplan übernehmen.</t>
         </is>
       </c>
     </row>
@@ -5380,7 +5376,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Von 46 Positionen tragen 46 einen Preis aus der API (22 über DigiKey, 24 über Mouser). Unter Vorbehalt: Vorschläge (Status gelb) sind noch nicht freigegeben, Positionen mit Status "Ersatz nötig" sind nicht ab Lager lieferbar.</t>
+          <t>Von 46 Positionen tragen 46 einen Preis aus der API (21 über DigiKey, 25 über Mouser). Unter Vorbehalt: Vorschläge (Status gelb) sind noch nicht freigegeben.</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5669,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>12401548E4-2A</t>
+          <t>12401598E4-2A</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -5693,7 +5689,7 @@
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>shbs_power:USB_C_Receptacle_Amphenol_12401548E4-2A</t>
+          <t>shbs_power:USB_C_Receptacle_Amphenol_12401598E4-2A</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
@@ -5703,10 +5699,14 @@
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>12401598E4#2A (Vorschlag)</t>
-        </is>
-      </c>
-      <c r="I7" s="16" t="inlineStr"/>
+          <t>12401598E4#2A</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>523-12401598E4#2A</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>12401548E4-2A</t>
+          <t>12401598E4-2A</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>shbs_power:USB_C_Receptacle_Amphenol_12401548E4-2A</t>
+          <t>shbs_power:USB_C_Receptacle_Amphenol_12401598E4-2A</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
@@ -6993,10 +6993,14 @@
       </c>
       <c r="H37" s="16" t="inlineStr">
         <is>
-          <t>12401598E4#2A (Vorschlag)</t>
-        </is>
-      </c>
-      <c r="I37" s="16" t="inlineStr"/>
+          <t>12401598E4#2A</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>523-12401598E4#2A</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -7324,19 +7328,15 @@
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>Monolithic Power Systems</t>
+          <t>Diodes Incorporated</t>
         </is>
       </c>
       <c r="H45" s="16" t="inlineStr">
         <is>
-          <t>MP2359DJ-LF-Z</t>
-        </is>
-      </c>
-      <c r="I45" s="16" t="inlineStr">
-        <is>
-          <t>946-MP2359DJ-LF-Z</t>
-        </is>
-      </c>
+          <t>AP3211KTR-G1 (Vorschlag)</t>
+        </is>
+      </c>
+      <c r="I45" s="16" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -8992,7 +8992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9056,17 +9056,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>1 abgekündigte Position</t>
+          <t>5 Positionen nur bei einem Anbieter</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>PS1 (MP2359DJ-LF-Z): Mouser Not Recommended for New Designs, Lager 0, DigiKey Nicht für Neukonstruktionen, Lager 0</t>
+          <t>C23 (nur Mouser); C25, C26 (nur Mouser); FB1 (nur DigiKey); R19, R20, R21, R22 (nur Mouser); S2 (nur Mouser)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Kein Beschaffungs-, sondern ein Abkündigungsproblem: auch ein Distributorwechsel hilft nicht. Ersatztyp wählen; hängt ein eigener Footprint daran, betrifft der Wechsel das Layout (Task 0041).</t>
+          <t>Kein Ausweichen möglich, falls der Anbieter ausverkauft ist. Beim Wechsel auf ein breiter verfügbares Teil den Footprint im Blick behalten.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -9081,17 +9081,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>5 Positionen nur bei einem Anbieter</t>
+          <t>30 Positionen mit Teilevorschlag</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>C23 (nur Mouser); C25, C26 (nur Mouser); FB1 (nur DigiKey); R19, R20, R21, R22 (nur Mouser); S2 (nur Mouser)</t>
+          <t>C13: CL21B106KOQNNNE; C14: CL21A226MOQNNNE; C15: CC0805KRX7R9BB104; C16, C17, C18, C19, C20, C21, C22: CC0805KRX7R9BB104; C23: CL21A475KAQNNNE; C24, C31: CC0805KRX7R9BB103; C25, C26: CC0805JRNPO9BN270; C27: CL21B106KOQNNNE; C28: C1206C102KGRACTU; C29, C30: CC0805KRX7R9BB682; C32: CL21B223KBANNNC; D8: 151033BS03000; D9: 151033RS03000; D10: 151031VS06000; F1: MF-NSMF110-2; FB1: BLM21PG601SN1D; PS1: AP3211KTR-G1; Q1, Q2, Q3, Q4: BC33740TA; R9: MFR-25FBF52-10K; R13, R14, R15, R16: PR02000202200JR500; R17: RC0805FR-0749K9L; R18: RC0805FR-0716K2L; R19, R20, R21, R22: RC0805FR-075K1L; R23, R24, R25, R26: PR02000204701JR500; R27: RC0805FR-0712K4L; R28, R29, R30, R31, R32: RC0805FR-0710KL; R33, R34: RC0805FR-07220RL; R35: RC0805JR-070RL; R36, R37, R39, R40: RC0805FR-0749R9L; R38: RC0805FR-0710RL</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Kein Ausweichen möglich, falls der Anbieter ausverkauft ist. Beim Wechsel auf ein breiter verfügbares Teil den Footprint im Blick behalten.</t>
+          <t>Der Schaltplan trägt hier nur einen Wert oder ein abgekündigtes Teil. Die Vorschläge folgen einem Hausstandard (Widerstände 0805 1 %, Kondensatoren X7R 50 V bzw. X5R/X7R 16–25 V ab 1 µF, C0G am Quarz) und sind in Spalte Status gelb markiert. Nach Freigabe als Felder in den Schaltplan übernehmen, damit der nächste Export sie ohne Skript-Tabelle trägt. J1/J_PWR1: Zeichnung des Nachfolgers vor der Übernahme gegen den Footprint prüfen.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -9106,17 +9106,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>30 Positionen mit Teilevorschlag</t>
+          <t>Abgeleitete Teilenummern</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>C13: CL21B106KOQNNNE; C14: CL21A226MOQNNNE; C15: CC0805KRX7R9BB104; C16, C17, C18, C19, C20, C21, C22: CC0805KRX7R9BB104; C23: CL21A475KAQNNNE; C24, C31: CC0805KRX7R9BB103; C25, C26: CC0805JRNPO9BN270; C27: CL21B106KOQNNNE; C28: C1206C102KGRACTU; C29, C30: CC0805KRX7R9BB682; C32: CL21B223KBANNNC; D8: 151033BS03000; D9: 151033RS03000; D10: 151031VS06000; F1: MF-NSMF110-2; FB1: BLM21PG601SN1D; J1, J_PWR1: 12401598E4#2A; Q1, Q2, Q3, Q4: BC33740TA; R9: MFR-25FBF52-10K; R13, R14, R15, R16: PR02000202200JR500; R17: RC0805FR-0749K9L; R18: RC0805FR-0716K2L; R19, R20, R21, R22: RC0805FR-075K1L; R23, R24, R25, R26: PR02000204701JR500; R27: RC0805FR-0712K4L; R28, R29, R30, R31, R32: RC0805FR-0710KL; R33, R34: RC0805FR-07220RL; R35: RC0805JR-070RL; R36, R37, R39, R40: RC0805FR-0749R9L; R38: RC0805FR-0710RL</t>
+          <t>Bei D11, D12, U1, L1 und J6 stammt die Nummer aus Wert oder Bibliotheksnamen, nicht aus einem gepflegten Feld.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Der Schaltplan trägt hier nur einen Wert oder ein abgekündigtes Teil. Die Vorschläge folgen einem Hausstandard (Widerstände 0805 1 %, Kondensatoren X7R 50 V bzw. X5R/X7R 16–25 V ab 1 µF, C0G am Quarz) und sind in Spalte Status gelb markiert. Nach Freigabe als Felder in den Schaltplan übernehmen, damit der nächste Export sie ohne Skript-Tabelle trägt. J1/J_PWR1: Zeichnung des Nachfolgers vor der Übernahme gegen den Footprint prüfen.</t>
+          <t>In der Spalte Status als "abgeleitet" markiert. Vor der Bestellung am Datenblatt bestätigen — Serienbezeichnungen wie SRN6045TA brauchen noch den Wert-Suffix.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -9131,22 +9131,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Abgeleitete Teilenummern</t>
+          <t>F1 (Sicherung)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Bei D11, D12, U1, L1 und J6 stammt die Nummer aus Wert oder Bibliotheksnamen, nicht aus einem gepflegten Feld.</t>
+          <t>Der Wert im Schaltplan lautet schlicht "Fuse" — kein Strom- oder Auslösewert.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>In der Spalte Status als "abgeleitet" markiert. Vor der Bestellung am Datenblatt bestätigen — Serienbezeichnungen wie SRN6045TA brauchen noch den Wert-Suffix.</t>
+          <t>Nennstrom steht in power_supply.md (Polyfuse 1,1 A); der Vorschlag MF-NSMF110-2 folgt dem. Den Wert auch im Schaltplan eintragen, sonst liest man dort nur "Fuse".</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Bediener</t>
+          <t>Agent</t>
         </is>
       </c>
     </row>
@@ -9156,17 +9156,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>F1 (Sicherung)</t>
+          <t>FB1 (Ferritperle)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Der Wert im Schaltplan lautet schlicht "Fuse" — kein Strom- oder Auslösewert.</t>
+          <t>Nutzt das Symbol Device:R — also einen Widerstand.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Nennstrom steht in power_supply.md (Polyfuse 1,1 A); der Vorschlag MF-NSMF110-2 folgt dem. Den Wert auch im Schaltplan eintragen, sonst liest man dort nur "Fuse".</t>
+          <t>Elektrisch folgenlos (zweipoliges Passivteil), aber Symbol und Bauteil widersprechen sich. Wer den Schaltplan liest, sieht einen Widerstand.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -9181,17 +9181,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>FB1 (Ferritperle)</t>
+          <t>J6 (Stiftleiste)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Nutzt das Symbol Device:R — also einen Widerstand.</t>
+          <t>Wert ist der generische KiCad-Symbolname "Conn_02x03_Odd_Even".</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Elektrisch folgenlos (zweipoliges Passivteil), aber Symbol und Bauteil widersprechen sich. Wer den Schaltplan liest, sieht einen Widerstand.</t>
+          <t>Der Footprint verweist auf Würth 61200621621. Der Wert sollte die Bestellbezeichnung tragen, sonst ist die Stückliste ohne Blick in den Footprint nicht lesbar.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -9206,22 +9206,22 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>J6 (Stiftleiste)</t>
+          <t>D8, D9, D10 (LEDs)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Wert ist der generische KiCad-Symbolname "Conn_02x03_Odd_Even".</t>
+          <t>Nutzen das generische Symbol Device:LED, während D7 das spezifische WL-TMRC_3MM-Symbol nutzt.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Der Footprint verweist auf Würth 61200621621. Der Wert sollte die Bestellbezeichnung tragen, sonst ist die Stückliste ohne Blick in den Footprint nicht lesbar.</t>
+          <t>Uneinheitlich. Zudem liegen D8/D9 auf der Serie WL-TMRW, D10 auf WL-TMRC — zwei verschiedene Würth-Serien in derselben Funktionsgruppe.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Agent</t>
+          <t>Bediener</t>
         </is>
       </c>
     </row>
@@ -9231,17 +9231,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>D8, D9, D10 (LEDs)</t>
+          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Nutzen das generische Symbol Device:LED, während D7 das spezifische WL-TMRC_3MM-Symbol nutzt.</t>
+          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Uneinheitlich. Zudem liegen D8/D9 auf der Serie WL-TMRW, D10 auf WL-TMRC — zwei verschiedene Würth-Serien in derselben Funktionsgruppe.</t>
+          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -9256,45 +9256,20 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
+          <t>Preise sind Tagespreise</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
+          <t>Die grün hinterlegten Einzelpreise stammen aus der Mouser- und der DigiKey-API zum Stand oben.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
+          <t>Sie sind unverbindlich, gelten für die Staffel passend zur Menge einer Baugruppe und verstehen sich ohne Zoll, Versand und Steuer. Für ein Angebot neu abfragen.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Bediener</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Preise sind Tagespreise</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Die grün hinterlegten Einzelpreise stammen aus der Mouser- und der DigiKey-API zum Stand oben.</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Sie sind unverbindlich, gelten für die Staffel passend zur Menge einer Baugruppe und verstehen sich ohne Zoll, Versand und Steuer. Für ein Angebot neu abfragen.</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Bediener</t>
         </is>

</xml_diff>

<commit_message>
v0.00.001 feat(SHBS-17): PS1 auf AP3211 umgestellt, V_FB-Formel in der Doku korrigiert
Der MP2359 ist in allen Varianten NRND und ohne Lager. Ersetzt durch den
pinkompatiblen Diodes AP3211KTR-G1 (SOT-23-6, V_FB 0,81 V, 1,4 MHz,
asynchron, 1,5 A). Symbol in shbs_power:AP3211 umbenannt, Felder in
Schaltplan und power.kicad_sym umgestellt; Footprint MP2359DJ passt
unveraendert. ERC 0 Fehler, Netzliste an PS1 unveraendert. L1-Saettigung
(4,6 A) gegen Strombegrenzung (max. 2,4 A) geprueft.

power_supply.md: V_OUT-Formel nannte 0,6 V statt 0,81 V.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
+++ b/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
@@ -3326,7 +3326,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>MP2359DJ</t>
+          <t>AP3211</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -3404,16 +3404,12 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="V32" s="10" t="inlineStr">
-        <is>
-          <t>Vorschlag</t>
-        </is>
-      </c>
-      <c r="W32" s="5" t="inlineStr">
-        <is>
-          <t>Ersatz für MP2359DJ-LF-Z (abgekündigt). Pinkompatibel (1 BS, 2 GND, 3 FB, 4 EN, 5 IN, 6 SW), SOT-23-6 passt auf den Footprint MP2359DJ, VFB 0,81 V (R17/R18 bleiben), 1,4 MHz, asynchron mit D11, 1,5 A. Prüfen: Strombegrenzung 1,8–2,4 A gegen den Sättigungsstrom von L1. Nach Freigabe als Feld in den Schaltplan übernehmen.</t>
-        </is>
-      </c>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -7303,7 +7299,7 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>MP2359DJ</t>
+          <t>AP3211</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
@@ -7318,14 +7314,14 @@
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
+          <t>shbs_power:AP3211</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
           <t>shbs_power:MP2359DJ</t>
         </is>
       </c>
-      <c r="F45" s="16" t="inlineStr">
-        <is>
-          <t>shbs_power:MP2359DJ</t>
-        </is>
-      </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
           <t>Diodes Incorporated</t>
@@ -7333,10 +7329,14 @@
       </c>
       <c r="H45" s="16" t="inlineStr">
         <is>
-          <t>AP3211KTR-G1 (Vorschlag)</t>
-        </is>
-      </c>
-      <c r="I45" s="16" t="inlineStr"/>
+          <t>AP3211KTR-G1</t>
+        </is>
+      </c>
+      <c r="I45" s="16" t="inlineStr">
+        <is>
+          <t>621-AP3211KTR-G1</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -9081,12 +9081,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>30 Positionen mit Teilevorschlag</t>
+          <t>29 Positionen mit Teilevorschlag</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>C13: CL21B106KOQNNNE; C14: CL21A226MOQNNNE; C15: CC0805KRX7R9BB104; C16, C17, C18, C19, C20, C21, C22: CC0805KRX7R9BB104; C23: CL21A475KAQNNNE; C24, C31: CC0805KRX7R9BB103; C25, C26: CC0805JRNPO9BN270; C27: CL21B106KOQNNNE; C28: C1206C102KGRACTU; C29, C30: CC0805KRX7R9BB682; C32: CL21B223KBANNNC; D8: 151033BS03000; D9: 151033RS03000; D10: 151031VS06000; F1: MF-NSMF110-2; FB1: BLM21PG601SN1D; PS1: AP3211KTR-G1; Q1, Q2, Q3, Q4: BC33740TA; R9: MFR-25FBF52-10K; R13, R14, R15, R16: PR02000202200JR500; R17: RC0805FR-0749K9L; R18: RC0805FR-0716K2L; R19, R20, R21, R22: RC0805FR-075K1L; R23, R24, R25, R26: PR02000204701JR500; R27: RC0805FR-0712K4L; R28, R29, R30, R31, R32: RC0805FR-0710KL; R33, R34: RC0805FR-07220RL; R35: RC0805JR-070RL; R36, R37, R39, R40: RC0805FR-0749R9L; R38: RC0805FR-0710RL</t>
+          <t>C13: CL21B106KOQNNNE; C14: CL21A226MOQNNNE; C15: CC0805KRX7R9BB104; C16, C17, C18, C19, C20, C21, C22: CC0805KRX7R9BB104; C23: CL21A475KAQNNNE; C24, C31: CC0805KRX7R9BB103; C25, C26: CC0805JRNPO9BN270; C27: CL21B106KOQNNNE; C28: C1206C102KGRACTU; C29, C30: CC0805KRX7R9BB682; C32: CL21B223KBANNNC; D8: 151033BS03000; D9: 151033RS03000; D10: 151031VS06000; F1: MF-NSMF110-2; FB1: BLM21PG601SN1D; Q1, Q2, Q3, Q4: BC33740TA; R9: MFR-25FBF52-10K; R13, R14, R15, R16: PR02000202200JR500; R17: RC0805FR-0749K9L; R18: RC0805FR-0716K2L; R19, R20, R21, R22: RC0805FR-075K1L; R23, R24, R25, R26: PR02000204701JR500; R27: RC0805FR-0712K4L; R28, R29, R30, R31, R32: RC0805FR-0710KL; R33, R34: RC0805FR-07220RL; R35: RC0805JR-070RL; R36, R37, R39, R40: RC0805FR-0749R9L; R38: RC0805FR-0710RL</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
v0.00.001 feat(SHBS-17): Abgeleitete Teilenummern bestaetigt und eingetragen, SHBS-17 abgeschlossen
D11 Comchip SS34-HF (SMA; die guenstigere Slkormicro-SS34 ist SMC und passt nicht auf D_SMA), D12 Littelfuse SMAJ5.0A, U1 D3V3XA4B10LP-7, L1 Bourns SRN6045TA-100M, J6 Wuerth 61200621621 als Felder im Schaltplan. DERIVED_PART_NUMBERS geleert. DigiKey-Stichwortsuche bevorzugt den Hersteller aus dem Schaltplan statt des billigsten Doppelgaengers. Netzliste identisch, ERC 0 Fehler. Stueckliste: 44 Positionen, alle eindeutig und lieferbar, 48,29 EUR. Task 0041 abgeschlossen; in Task 0042 zwei durch SHBS-17 erledigte Schritte vermerkt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
+++ b/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
@@ -2370,35 +2370,35 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Shenzhen Slkormicro Semicon Co., Ltd.</t>
+          <t>Comchip Technology</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>SS34</t>
+          <t>SS34-HF</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>512-SS34</t>
+          <t>750-SS34-HF</t>
         </is>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.869</v>
+        <v>0.464</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>57173</v>
+        <v>22099</v>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>5399-SS34CT-ND</t>
+          <t>641-2115-1-ND</t>
         </is>
       </c>
       <c r="M23" s="7" t="n">
-        <v>0.13</v>
+        <v>0.46</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>8977</v>
+        <v>53701</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
@@ -2435,14 +2435,10 @@
       </c>
       <c r="V23" s="4" t="inlineStr">
         <is>
-          <t>abgeleitet</t>
-        </is>
-      </c>
-      <c r="W23" s="5" t="inlineStr">
-        <is>
-          <t>Teilenummer aus Wert/Bibliothek abgeleitet — am Datenblatt bestätigen.</t>
-        </is>
-      </c>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -2473,7 +2469,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Shenzhen Slkormicro Semicon Co., Ltd.</t>
+          <t>Littelfuse</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2483,25 +2479,25 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>78-SMAJ5.0A</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="n">
-        <v>0.387</v>
+          <t>576-SMAJ5.0A</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>0.378</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>3173</v>
+        <v>24547</v>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>5399-SMAJ5.0ACT-ND</t>
-        </is>
-      </c>
-      <c r="M24" s="7" t="n">
-        <v>0.2</v>
+          <t>SMAJ5.0ALFCT-ND</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>0.43</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>35768</v>
+        <v>167866</v>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
@@ -2510,7 +2506,7 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q24" s="8">
@@ -2538,14 +2534,10 @@
       </c>
       <c r="V24" s="4" t="inlineStr">
         <is>
-          <t>abgeleitet</t>
-        </is>
-      </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>Teilenummer aus Wert/Bibliothek abgeleitet — am Datenblatt bestätigen.</t>
-        </is>
-      </c>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2894,7 +2886,7 @@
         <v>0.404</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>47078</v>
+        <v>46778</v>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
@@ -2942,14 +2934,10 @@
       </c>
       <c r="V28" s="4" t="inlineStr">
         <is>
-          <t>abgeleitet</t>
-        </is>
-      </c>
-      <c r="W28" s="5" t="inlineStr">
-        <is>
-          <t>Teilenummer aus Wert/Bibliothek abgeleitet — am Datenblatt bestätigen.</t>
-        </is>
-      </c>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -2997,7 +2985,7 @@
         <v>0.43</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>4322</v>
+        <v>4297</v>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
@@ -3045,14 +3033,10 @@
       </c>
       <c r="V29" s="4" t="inlineStr">
         <is>
-          <t>abgeleitet</t>
-        </is>
-      </c>
-      <c r="W29" s="5" t="inlineStr">
-        <is>
-          <t>Teilenummer aus Wert/Bibliothek abgeleitet — am Datenblatt bestätigen.</t>
-        </is>
-      </c>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -4664,7 +4648,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>D3V3XA4B10LP</t>
+          <t>D3V3XA4B10LP-7</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -4724,14 +4708,10 @@
       </c>
       <c r="V46" s="4" t="inlineStr">
         <is>
-          <t>abgeleitet</t>
-        </is>
-      </c>
-      <c r="W46" s="5" t="inlineStr">
-        <is>
-          <t>Teilenummer aus Wert/Bibliothek abgeleitet — am Datenblatt bestätigen.</t>
-        </is>
-      </c>
+          <t>eindeutig</t>
+        </is>
+      </c>
+      <c r="W46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -5066,7 +5046,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Von 44 Positionen tragen 44 einen Preis aus der API (20 über DigiKey, 24 über Mouser). </t>
+          <t xml:space="preserve">Von 44 Positionen tragen 44 einen Preis aus der API (19 über DigiKey, 25 über Mouser). </t>
         </is>
       </c>
     </row>
@@ -5434,10 +5414,14 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>D3V3XA4B10LP</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr"/>
+          <t>D3V3XA4B10LP-7</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>621-D3V3XA4B10LP-7</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -6525,7 +6509,11 @@
           <t>61200621621</t>
         </is>
       </c>
-      <c r="I32" s="15" t="inlineStr"/>
+      <c r="I32" s="15" t="inlineStr">
+        <is>
+          <t>710-61200621621</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
@@ -6840,13 +6828,21 @@
           <t>Diode_SMD:D_SMA</t>
         </is>
       </c>
-      <c r="G39" s="15" t="inlineStr"/>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>Comchip Technology</t>
+        </is>
+      </c>
       <c r="H39" s="15" t="inlineStr">
         <is>
-          <t>SS34</t>
-        </is>
-      </c>
-      <c r="I39" s="15" t="inlineStr"/>
+          <t>SS34-HF</t>
+        </is>
+      </c>
+      <c r="I39" s="15" t="inlineStr">
+        <is>
+          <t>750-SS34-HF</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
@@ -7067,13 +7063,21 @@
           <t>Diode_SMD:D_SMA</t>
         </is>
       </c>
-      <c r="G44" s="15" t="inlineStr"/>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>Littelfuse</t>
+        </is>
+      </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
           <t>SMAJ5.0A</t>
         </is>
       </c>
-      <c r="I44" s="15" t="inlineStr"/>
+      <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>576-SMAJ5.0A</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
@@ -7210,7 +7214,11 @@
           <t>SRN6045TA-100M</t>
         </is>
       </c>
-      <c r="I47" s="15" t="inlineStr"/>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>652-SRN6045TA-100M</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
@@ -8912,7 +8920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9001,22 +9009,22 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Abgeleitete Teilenummern</t>
+          <t>FB1 (Ferritperle)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Bei D11, D12, U1, L1 und J6 stammt die Nummer aus Wert oder Bibliotheksnamen, nicht aus einem gepflegten Feld.</t>
+          <t>Nutzt das Symbol Device:R — also einen Widerstand.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>In der Spalte Status als "abgeleitet" markiert. Vor der Bestellung am Datenblatt bestätigen — Serienbezeichnungen wie SRN6045TA brauchen noch den Wert-Suffix.</t>
+          <t>Elektrisch folgenlos (zweipoliges Passivteil), aber Symbol und Bauteil widersprechen sich. Wer den Schaltplan liest, sieht einen Widerstand.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Bediener</t>
+          <t>Agent</t>
         </is>
       </c>
     </row>
@@ -9026,17 +9034,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>FB1 (Ferritperle)</t>
+          <t>J6 (Stiftleiste)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Nutzt das Symbol Device:R — also einen Widerstand.</t>
+          <t>Wert ist der generische KiCad-Symbolname "Conn_02x03_Odd_Even".</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Elektrisch folgenlos (zweipoliges Passivteil), aber Symbol und Bauteil widersprechen sich. Wer den Schaltplan liest, sieht einen Widerstand.</t>
+          <t>Der Footprint verweist auf Würth 61200621621. Der Wert sollte die Bestellbezeichnung tragen, sonst ist die Stückliste ohne Blick in den Footprint nicht lesbar.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -9051,22 +9059,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>J6 (Stiftleiste)</t>
+          <t>D8, D9, D10 (LEDs)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Wert ist der generische KiCad-Symbolname "Conn_02x03_Odd_Even".</t>
+          <t>Nutzen das generische Symbol Device:LED, während D7 das spezifische WL-TMRC_3MM-Symbol nutzt.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Der Footprint verweist auf Würth 61200621621. Der Wert sollte die Bestellbezeichnung tragen, sonst ist die Stückliste ohne Blick in den Footprint nicht lesbar.</t>
+          <t>Uneinheitlich. Zudem liegen D8/D9 auf der Serie WL-TMRW, D10 auf WL-TMRC — zwei verschiedene Würth-Serien in derselben Funktionsgruppe.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Agent</t>
+          <t>Bediener</t>
         </is>
       </c>
     </row>
@@ -9076,17 +9084,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>D8, D9, D10 (LEDs)</t>
+          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Nutzen das generische Symbol Device:LED, während D7 das spezifische WL-TMRC_3MM-Symbol nutzt.</t>
+          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Uneinheitlich. Zudem liegen D8/D9 auf der Serie WL-TMRW, D10 auf WL-TMRC — zwei verschiedene Würth-Serien in derselben Funktionsgruppe.</t>
+          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -9101,45 +9109,20 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
+          <t>Preise sind Tagespreise</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
+          <t>Die grün hinterlegten Einzelpreise stammen aus der Mouser- und der DigiKey-API zum Stand oben.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
+          <t>Sie sind unverbindlich, gelten für die Staffel passend zur Menge einer Baugruppe und verstehen sich ohne Zoll, Versand und Steuer. Für ein Angebot neu abfragen.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Bediener</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Preise sind Tagespreise</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Die grün hinterlegten Einzelpreise stammen aus der Mouser- und der DigiKey-API zum Stand oben.</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Sie sind unverbindlich, gelten für die Staffel passend zur Menge einer Baugruppe und verstehen sich ohne Zoll, Versand und Steuer. Für ein Angebot neu abfragen.</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Bediener</t>
         </is>

</xml_diff>

<commit_message>
v0.00.001 fix(SHBS-16): D10-Verpolung behoben, LED-Symbole vereinheitlicht, FB1 und J6 bereinigt
Footprint WL-TMRC_3MM hatte Pad 1 = Anode, Device:LED hat Pin 1 = Kathode: D10 lag mit der Kathode an +3V3 und haette nie geleuchtet. Footprint auf Pad 1 = K / Pad 2 = A umnummeriert (wie WL-TMRW_3MM), Wuerth-Symbol mitgezogen. D7 von WL-TMRC_3MM auf Device:LED, so platziert, dass K/A auf den bisherigen Drahtenden liegen. FB1 auf Device:FerriteBead, J6-Wert auf 61200621621.

Gegenprobe: ERC 0 Fehler; Netzliste mit gleichen Bauteilen je Netz, nur D7-Pinnummern getauscht; Polaritaet aller vier LEDs auf Pad-Ebene geprueft. Beim naechsten PCB-Abgleich Footprint von D7/D10 aus der Bibliothek aktualisieren. Task 0042 abgeschlossen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
+++ b/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
@@ -2854,7 +2854,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Conn_02x03_Odd_Even</t>
+          <t>61200621621</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>WL-TMRC_3MM:WL-TMRC_3MM</t>
+          <t>Device:LED</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Conn_02x03_Odd_Even</t>
+          <t>61200621621</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:FerriteBead</t>
         </is>
       </c>
       <c r="F52" s="15" t="inlineStr">
@@ -8920,7 +8920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9009,22 +9009,22 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>FB1 (Ferritperle)</t>
+          <t>D7–D10 (LEDs): zwei Würth-Serien</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Nutzt das Symbol Device:R — also einen Widerstand.</t>
+          <t>D7/D10 sind WL-TMRC (eingefärbt, diffus), D8/D9 WL-TMRW (wasserklar).</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Elektrisch folgenlos (zweipoliges Passivteil), aber Symbol und Bauteil widersprechen sich. Wer den Schaltplan liest, sieht einen Widerstand.</t>
+          <t>Elektrisch gleichwertig, optisch nicht: wasserklare LEDs strahlen gerichteter und wirken bei gleichem Strom heller. Für ein einheitliches Erscheinungsbild eine Serie wählen — beide Footprints sind seit SHBS-16 gleich nummeriert (1 = K, 2 = A).</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Agent</t>
+          <t>Bediener</t>
         </is>
       </c>
     </row>
@@ -9034,22 +9034,22 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>J6 (Stiftleiste)</t>
+          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Wert ist der generische KiCad-Symbolname "Conn_02x03_Odd_Even".</t>
+          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Der Footprint verweist auf Würth 61200621621. Der Wert sollte die Bestellbezeichnung tragen, sonst ist die Stückliste ohne Blick in den Footprint nicht lesbar.</t>
+          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Agent</t>
+          <t>Bediener</t>
         </is>
       </c>
     </row>
@@ -9059,70 +9059,20 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>D8, D9, D10 (LEDs)</t>
+          <t>Preise sind Tagespreise</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Nutzen das generische Symbol Device:LED, während D7 das spezifische WL-TMRC_3MM-Symbol nutzt.</t>
+          <t>Die grün hinterlegten Einzelpreise stammen aus der Mouser- und der DigiKey-API zum Stand oben.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Uneinheitlich. Zudem liegen D8/D9 auf der Serie WL-TMRW, D10 auf WL-TMRC — zwei verschiedene Würth-Serien in derselben Funktionsgruppe.</t>
+          <t>Sie sind unverbindlich, gelten für die Staffel passend zur Menge einer Baugruppe und verstehen sich ohne Zoll, Versand und Steuer. Für ein Angebot neu abfragen.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Bediener</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Bediener</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Preise sind Tagespreise</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Die grün hinterlegten Einzelpreise stammen aus der Mouser- und der DigiKey-API zum Stand oben.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Sie sind unverbindlich, gelten für die Staffel passend zur Menge einer Baugruppe und verstehen sich ohne Zoll, Versand und Steuer. Für ein Angebot neu abfragen.</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Bediener</t>
         </is>

</xml_diff>

<commit_message>
v0.00.001 fix(SHBS-17): Q1-Q4 auf BC33740BU mit geraden Beinen, TA-Variante passte nicht auf TO-92_Inline
Die Gurt-Variante BC33740TA hat auf 2,54 mm aufgebogene Anschlussbeine, der Footprint TO-92_Inline hat 1,27 mm Raster. Umgestellt auf onsemi BC33740BU (gleiches Datenblatt, gerade Beine, Pinbelegung C-B-E unveraendert). Beim systematischen Footprint-Abgleich aufgefallen: alle anderen 72 Bauteile passen zu ihrem Footprint.

Gegenprobe: Netzliste identisch, Stueckliste 44 Positionen eindeutig und lieferbar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
+++ b/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
@@ -538,7 +538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-23 · 44 Positionen · 78 Bauteile</t>
+          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-24 · 44 Positionen · 78 Bauteile</t>
         </is>
       </c>
     </row>
@@ -3171,30 +3171,30 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>BC33740TA</t>
+          <t>BC33740BU</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>512-BC33740TA</t>
+          <t>512-BC33740BU</t>
         </is>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.258</v>
+        <v>0.249</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>18419</v>
+        <v>22995</v>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>BC33740TACT-ND</t>
+          <t>BC33740BU-ND</t>
         </is>
       </c>
       <c r="M31" s="6" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>1274</v>
+        <v>2763</v>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
@@ -5224,7 +5224,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alle 78 bestückten Referenzen einzeln · Stand 2026-09-23</t>
+          <t>Alle 78 bestückten Referenzen einzeln · Stand 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -5508,12 +5508,12 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>BC33740TA</t>
+          <t>BC33740BU</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740TA</t>
+          <t>512-BC33740BU</t>
         </is>
       </c>
     </row>
@@ -5813,12 +5813,12 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>BC33740TA</t>
+          <t>BC33740BU</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740TA</t>
+          <t>512-BC33740BU</t>
         </is>
       </c>
     </row>
@@ -6275,12 +6275,12 @@
       </c>
       <c r="H27" s="15" t="inlineStr">
         <is>
-          <t>BC33740TA</t>
+          <t>BC33740BU</t>
         </is>
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740TA</t>
+          <t>512-BC33740BU</t>
         </is>
       </c>
     </row>
@@ -6600,12 +6600,12 @@
       </c>
       <c r="H34" s="15" t="inlineStr">
         <is>
-          <t>BC33740TA</t>
+          <t>BC33740BU</t>
         </is>
       </c>
       <c r="I34" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740TA</t>
+          <t>512-BC33740BU</t>
         </is>
       </c>
     </row>
@@ -8940,7 +8940,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stand 2026-09-23 · Der Schaltplan ist elektrisch fertig (ERC 0 Fehler).</t>
+          <t>Stand 2026-09-24 · Der Schaltplan ist elektrisch fertig (ERC 0 Fehler).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.00.001 docs(SHBS-17): Stueckliste mit aktuellen Tagespreisen, U6 fest ueber Mouser
Alle Preise und Lagerbestaende per --refresh neu abgefragt. U7 wechselt dadurch zu Mouser, C32 zu DigiKey. U6 (ESP32-S3-WROOM-1U-N16R8) auf Wunsch des Bedieners fest ueber Mouser: DigiKey hat nur noch 66 Stueck, Mouser rund 6100, Aufpreis 0,14 EUR. Die Festlegung steht mit Begruendung in SOURCE_OVERRIDES und erscheint in der Hinweisspalte. Summe 48,40 EUR pro Baugruppe (DigiKey 28,45, Mouser 19,95).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
+++ b/tmp/report/2026-09-22_stueckliste-basisstation.xlsx
@@ -1004,7 +1004,7 @@
         <v>1.35</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>1267</v>
+        <v>1017</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0.344</v>
+        <v>0.421</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>328250</v>
+        <v>323680</v>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
         <v>0.24</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>334334</v>
+        <v>277103</v>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
         <v>0.27</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>31248</v>
+        <v>25218</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
         <v>0.12</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>978450</v>
+        <v>1217786</v>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
         <v>0.15</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1635533</v>
+        <v>1635243</v>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="M13" s="6" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="N13" s="10" t="n">
         <v>0</v>
@@ -1492,7 +1492,7 @@
         <v>0.146</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>359008</v>
+        <v>358983</v>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
         <v>0.12</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>238857</v>
+        <v>234857</v>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         <v>1.33</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>196525</v>
+        <v>196492</v>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
@@ -1705,7 +1705,7 @@
         <v>1.33</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>605538</v>
+        <v>605024</v>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>0.12</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>1640</v>
+        <v>1630</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -1888,22 +1888,22 @@
           <t>187-CL21B223KBANNNC</t>
         </is>
       </c>
-      <c r="J18" s="7" t="n">
-        <v>0.08599999999999999</v>
+      <c r="J18" s="6" t="n">
+        <v>0.138</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>3172</v>
+        <v>3047</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
           <t>1276-1081-1-ND</t>
         </is>
       </c>
-      <c r="M18" s="6" t="n">
+      <c r="M18" s="7" t="n">
         <v>0.09</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>9535</v>
+        <v>9435</v>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Mouser</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="Q18" s="8">
@@ -2189,7 +2189,7 @@
         <v>0.146</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>34377</v>
+        <v>34357</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
         <v>0.14</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>53498</v>
+        <v>53301</v>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
         <v>0.378</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>24547</v>
+        <v>24423</v>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
         <v>0.43</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>167866</v>
+        <v>167714</v>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
@@ -2695,7 +2695,7 @@
         <v>0.1</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>4801</v>
+        <v>4446</v>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
         <v>0.43</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>21047</v>
+        <v>20950</v>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
@@ -2996,7 +2996,7 @@
         <v>0.43</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>4364</v>
+        <v>4355</v>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
@@ -3282,7 +3282,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>129072</v>
+        <v>128848</v>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
@@ -3293,7 +3293,7 @@
         <v>0.09</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>90754</v>
+        <v>89882</v>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>196225</v>
+        <v>195715</v>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
@@ -3491,7 +3491,7 @@
         <v>0.09</v>
       </c>
       <c r="N34" s="4" t="n">
-        <v>950285</v>
+        <v>950283</v>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         <v>0.103</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>41518</v>
+        <v>36518</v>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
@@ -3880,7 +3880,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>9850</v>
+        <v>9810</v>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
@@ -3979,7 +3979,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>3468997</v>
+        <v>3453672</v>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
@@ -3990,7 +3990,7 @@
         <v>0.09</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>1962322</v>
+        <v>1935589</v>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
@@ -4078,7 +4078,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>218904</v>
+        <v>218894</v>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v>0.09</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>394529</v>
+        <v>380504</v>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
@@ -4177,7 +4177,7 @@
         <v>0.215</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>2670154</v>
+        <v>2669469</v>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
@@ -4188,7 +4188,7 @@
         <v>0.09</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>2866267</v>
+        <v>2861448</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>308194</v>
+        <v>308094</v>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
@@ -4287,7 +4287,7 @@
         <v>0.09</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>391340</v>
+        <v>376340</v>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
@@ -4375,7 +4375,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>124309</v>
+        <v>119285</v>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
@@ -4386,7 +4386,7 @@
         <v>0.1</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>602162</v>
+        <v>601024</v>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
@@ -4572,7 +4572,7 @@
         <v>5.92</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>2678</v>
+        <v>2673</v>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
@@ -4759,7 +4759,7 @@
         <v>5.93</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>6174</v>
+        <v>6109</v>
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
@@ -4770,7 +4770,7 @@
         <v>5.79</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q47" s="8">
@@ -4810,7 +4810,11 @@
           <t>eindeutig</t>
         </is>
       </c>
-      <c r="W47" s="5" t="inlineStr"/>
+      <c r="W47" s="5" t="inlineStr">
+        <is>
+          <t>Bezugsquelle Mouser festgelegt (Bediener, 2026-09-24): DigiKey hat nur zweistelligen Lagerbestand, Mouser mehrere Tausend — sicherer fuer groessere Stueckzahlen, Aufpreis rund 0,14 EUR.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -4854,22 +4858,22 @@
           <t>950-W5500</t>
         </is>
       </c>
-      <c r="J48" s="6" t="n">
+      <c r="J48" s="7" t="n">
         <v>2.98</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>43647</v>
+        <v>43173</v>
       </c>
       <c r="L48" s="4" t="inlineStr">
         <is>
           <t>1278-W5500CT-ND</t>
         </is>
       </c>
-      <c r="M48" s="7" t="n">
-        <v>2.97</v>
+      <c r="M48" s="6" t="n">
+        <v>3.18</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>62872</v>
+        <v>62550</v>
       </c>
       <c r="O48" s="4" t="inlineStr">
         <is>
@@ -4878,7 +4882,7 @@
       </c>
       <c r="P48" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q48" s="8">
@@ -5046,7 +5050,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Von 44 Positionen tragen 44 einen Preis aus der API (19 über DigiKey, 25 über Mouser). </t>
+          <t xml:space="preserve">Von 44 Positionen tragen 44 einen Preis aus der API (18 über DigiKey, 26 über Mouser). </t>
         </is>
       </c>
     </row>

</xml_diff>